<commit_message>
Working on a viable planting_name variable for plantings table.
</commit_message>
<xml_diff>
--- a/output_tables/archive/p_gps_pts1_groupno_old.xlsx
+++ b/output_tables/archive/p_gps_pts1_groupno_old.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://stateofwa-my.sharepoint.com/personal/peter_dowty_dnr_wa_gov/Documents/projects/seagrass_restoration_data_2026/output_tables/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://stateofwa-my.sharepoint.com/personal/peter_dowty_dnr_wa_gov/Documents/projects/seagrass_restoration_data_2026/output_tables/archive/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="49" documentId="8_{8D93D302-86F1-4BDE-BA85-C1D4E21B1AFC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{02FD3076-BE1A-4882-BE07-28896B30D63A}"/>
+  <xr:revisionPtr revIDLastSave="50" documentId="8_{8D93D302-86F1-4BDE-BA85-C1D4E21B1AFC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7504AB74-7A8C-41D1-B1D4-8A0E80DFE196}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="45" windowWidth="28785" windowHeight="15390" xr2:uid="{308FDB03-57E4-4B58-ADF4-6D420AFE65D3}"/>
+    <workbookView xWindow="0" yWindow="30" windowWidth="28800" windowHeight="15360" xr2:uid="{308FDB03-57E4-4B58-ADF4-6D420AFE65D3}"/>
   </bookViews>
   <sheets>
     <sheet name="p_gps_pts1_groupno" sheetId="1" r:id="rId1"/>
@@ -2782,10 +2782,6 @@
 </styleSheet>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -3111,32 +3107,32 @@
     <col min="3" max="3" width="59.28515625" customWidth="1"/>
     <col min="4" max="4" width="22" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="21.140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="5" hidden="1" customWidth="1"/>
-    <col min="7" max="7" width="225.140625" hidden="1" customWidth="1"/>
+    <col min="6" max="6" width="5" customWidth="1"/>
+    <col min="7" max="7" width="225.140625" customWidth="1"/>
     <col min="8" max="8" width="17.42578125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="20.7109375" hidden="1" customWidth="1"/>
-    <col min="10" max="10" width="12.140625" hidden="1" customWidth="1"/>
+    <col min="9" max="9" width="20.7109375" customWidth="1"/>
+    <col min="10" max="10" width="12.140625" customWidth="1"/>
     <col min="11" max="11" width="11.5703125" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="12" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="13.140625" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="12" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="12.7109375" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="11.140625" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="7" hidden="1" customWidth="1"/>
-    <col min="18" max="18" width="17.7109375" hidden="1" customWidth="1"/>
+    <col min="17" max="17" width="7" customWidth="1"/>
+    <col min="18" max="18" width="17.7109375" customWidth="1"/>
     <col min="19" max="19" width="16" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="16.85546875" hidden="1" customWidth="1"/>
-    <col min="21" max="21" width="22.7109375" hidden="1" customWidth="1"/>
-    <col min="22" max="22" width="12.85546875" hidden="1" customWidth="1"/>
-    <col min="23" max="23" width="16.28515625" hidden="1" customWidth="1"/>
-    <col min="24" max="24" width="24.5703125" hidden="1" customWidth="1"/>
-    <col min="25" max="25" width="21.7109375" hidden="1" customWidth="1"/>
-    <col min="26" max="26" width="14.85546875" hidden="1" customWidth="1"/>
-    <col min="27" max="27" width="21.42578125" hidden="1" customWidth="1"/>
-    <col min="28" max="28" width="29.85546875" hidden="1" customWidth="1"/>
+    <col min="20" max="20" width="16.85546875" customWidth="1"/>
+    <col min="21" max="21" width="22.7109375" customWidth="1"/>
+    <col min="22" max="22" width="12.85546875" customWidth="1"/>
+    <col min="23" max="23" width="16.28515625" customWidth="1"/>
+    <col min="24" max="24" width="24.5703125" customWidth="1"/>
+    <col min="25" max="25" width="21.7109375" customWidth="1"/>
+    <col min="26" max="26" width="14.85546875" customWidth="1"/>
+    <col min="27" max="27" width="21.42578125" customWidth="1"/>
+    <col min="28" max="28" width="29.85546875" customWidth="1"/>
     <col min="29" max="29" width="29.85546875" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="255.7109375" hidden="1" customWidth="1"/>
-    <col min="31" max="31" width="36" hidden="1" customWidth="1"/>
+    <col min="30" max="30" width="255.7109375" customWidth="1"/>
+    <col min="31" max="31" width="36" customWidth="1"/>
     <col min="32" max="32" width="9.28515625" bestFit="1" customWidth="1"/>
     <col min="33" max="33" width="16.7109375" customWidth="1"/>
     <col min="34" max="35" width="17.85546875" customWidth="1"/>

</xml_diff>